<commit_message>
[Add] Thêm chức năng import excel
</commit_message>
<xml_diff>
--- a/Users.xlsx
+++ b/Users.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Flutter\New folder\Face-Detection-with-Name-Recognition\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Face-Detection-with-Name-Recognition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDFFC50-B05F-44CF-BF01-8153D19859F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="2535" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="348" yWindow="2532" windowWidth="21600" windowHeight="11388"/>
   </bookViews>
   <sheets>
     <sheet name="Ý tooi là tạo bản exel như thế" sheetId="1" r:id="rId1"/>
@@ -37,9 +36,6 @@
     <t>password</t>
   </si>
   <si>
-    <t>student_id</t>
-  </si>
-  <si>
     <t>class_name</t>
   </si>
   <si>
@@ -113,12 +109,15 @@
   </si>
   <si>
     <t>student6@school.edu</t>
+  </si>
+  <si>
+    <t>student_code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -380,14 +379,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -404,118 +403,118 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="1" t="s">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="F4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="1" t="s">
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C6" r:id="rId1" xr:uid="{36921699-132D-4665-8797-934E0A2EE5AC}"/>
+    <hyperlink ref="C6" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>